<commit_message>
Add Programs template, generic sidenav block and BBA Major page importers
- Generic sidenav block: nested bulleted links, current-page detection, mobile disclosure
- Programs template: adds the shared Programs sidenav fragment beside page content
- Hero (caption) and Columns (red) variants, aside section style, SFU accordion styling
- Importers for /programs, /fragments/programs-sidenav, /templates/programs; block library entries

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/tools/importer/reports/import-block-library.report.xlsx
+++ b/tools/importer/reports/import-block-library.report.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="52" uniqueCount="30">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="79" uniqueCount="42">
   <si>
     <t>_reportFile</t>
   </si>
@@ -52,7 +52,7 @@
     <t>success</t>
   </si>
   <si>
-    <t>2026-10-28T07:35:18.301Z</t>
+    <t>2026-10-29T00:30:29.725Z</t>
   </si>
   <si>
     <t>https://www.sfu.ca/</t>
@@ -91,6 +91,30 @@
     <t>2026-10-28T07:28:21.326Z</t>
   </si>
   <si>
+    <t>programs.report.json</t>
+  </si>
+  <si>
+    <t>programs</t>
+  </si>
+  <si>
+    <t>2026-10-29T00:30:01.315Z</t>
+  </si>
+  <si>
+    <t>https://www.sfu.ca/beedie/programs/undergraduate/bba-major/program.html</t>
+  </si>
+  <si>
+    <t>fragments/programs-sidenav.report.json</t>
+  </si>
+  <si>
+    <t>fragments/programs-sidenav</t>
+  </si>
+  <si>
+    <t>programs-sidenav</t>
+  </si>
+  <si>
+    <t>2026-10-29T00:30:10.251Z</t>
+  </si>
+  <si>
     <t>templates/landing-page.report.json</t>
   </si>
   <si>
@@ -101,6 +125,18 @@
   </si>
   <si>
     <t>2026-10-28T07:31:46.139Z</t>
+  </si>
+  <si>
+    <t>templates/programs.report.json</t>
+  </si>
+  <si>
+    <t>templates/programs</t>
+  </si>
+  <si>
+    <t>programs-template</t>
+  </si>
+  <si>
+    <t>2026-10-29T00:30:19.873Z</t>
   </si>
 </sst>
 </file>
@@ -489,16 +525,16 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:I6"/>
+  <dimension ref="A1:I9"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
-    <col min="1" max="1" width="36" customWidth="1"/>
-    <col min="3" max="3" width="24" customWidth="1"/>
+    <col min="1" max="1" width="40" customWidth="1"/>
+    <col min="3" max="3" width="28" customWidth="1"/>
     <col min="4" max="4" width="10" customWidth="1"/>
-    <col min="6" max="6" width="15" customWidth="1"/>
+    <col min="6" max="6" width="19" customWidth="1"/>
     <col min="7" max="7" width="26" customWidth="1"/>
     <col min="8" max="8" width="25" customWidth="1"/>
-    <col min="9" max="9" width="21" customWidth="1"/>
+    <col min="9" max="9" width="50" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:9" s="1" customFormat="1" x14ac:dyDescent="0.25">
@@ -535,7 +571,7 @@
         <v>9</v>
       </c>
       <c r="B2">
-        <v>12</v>
+        <v>17</v>
       </c>
       <c r="C2" t="s">
         <v>10</v>
@@ -663,16 +699,103 @@
         <v>12</v>
       </c>
       <c r="F6" t="s">
+        <v>27</v>
+      </c>
+      <c r="G6" t="s">
         <v>28</v>
       </c>
-      <c r="G6" t="s">
+      <c r="H6" t="s">
+        <v>11</v>
+      </c>
+      <c r="I6" t="s">
         <v>29</v>
       </c>
-      <c r="H6" t="s">
-        <v>11</v>
-      </c>
-      <c r="I6" t="s">
+    </row>
+    <row r="7" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>30</v>
+      </c>
+      <c r="B7" t="s">
+        <v>11</v>
+      </c>
+      <c r="C7" t="s">
+        <v>31</v>
+      </c>
+      <c r="D7" t="s">
+        <v>11</v>
+      </c>
+      <c r="E7" t="s">
+        <v>12</v>
+      </c>
+      <c r="F7" t="s">
+        <v>32</v>
+      </c>
+      <c r="G7" t="s">
+        <v>33</v>
+      </c>
+      <c r="H7" t="s">
+        <v>11</v>
+      </c>
+      <c r="I7" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="8" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>34</v>
+      </c>
+      <c r="B8" t="s">
+        <v>11</v>
+      </c>
+      <c r="C8" t="s">
+        <v>35</v>
+      </c>
+      <c r="D8" t="s">
+        <v>11</v>
+      </c>
+      <c r="E8" t="s">
+        <v>12</v>
+      </c>
+      <c r="F8" t="s">
+        <v>36</v>
+      </c>
+      <c r="G8" t="s">
+        <v>37</v>
+      </c>
+      <c r="H8" t="s">
+        <v>11</v>
+      </c>
+      <c r="I8" t="s">
         <v>14</v>
+      </c>
+    </row>
+    <row r="9" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>38</v>
+      </c>
+      <c r="B9" t="s">
+        <v>11</v>
+      </c>
+      <c r="C9" t="s">
+        <v>39</v>
+      </c>
+      <c r="D9" t="s">
+        <v>11</v>
+      </c>
+      <c r="E9" t="s">
+        <v>12</v>
+      </c>
+      <c r="F9" t="s">
+        <v>40</v>
+      </c>
+      <c r="G9" t="s">
+        <v>41</v>
+      </c>
+      <c r="H9" t="s">
+        <v>11</v>
+      </c>
+      <c r="I9" t="s">
+        <v>29</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Add Resources template, Research Facilities page and Supabase-backed facilities block
- Shared sidenav layout used by the Programs and Resources templates
- Resources template with its own navigation fragment (generic sidenav block)
- facilities block: category dropdown from Supabase, filtered query per category
- scripts/supabase-config.js: browser-safe connection settings (publishable key to be added)
- Importers for /resources/research-facilities, /fragments/resources-sidenav, /templates/resources; block library entry

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/tools/importer/reports/import-block-library.report.xlsx
+++ b/tools/importer/reports/import-block-library.report.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="79" uniqueCount="42">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="106" uniqueCount="55">
   <si>
     <t>_reportFile</t>
   </si>
@@ -52,7 +52,7 @@
     <t>success</t>
   </si>
   <si>
-    <t>2026-10-29T00:30:29.725Z</t>
+    <t>2026-10-29T00:58:57.058Z</t>
   </si>
   <si>
     <t>https://www.sfu.ca/</t>
@@ -97,7 +97,7 @@
     <t>programs</t>
   </si>
   <si>
-    <t>2026-10-29T00:30:01.315Z</t>
+    <t>2026-10-29T00:49:24.817Z</t>
   </si>
   <si>
     <t>https://www.sfu.ca/beedie/programs/undergraduate/bba-major/program.html</t>
@@ -112,7 +112,34 @@
     <t>programs-sidenav</t>
   </si>
   <si>
-    <t>2026-10-29T00:30:10.251Z</t>
+    <t>2026-10-29T00:31:18.120Z</t>
+  </si>
+  <si>
+    <t>fragments/resources-sidenav.report.json</t>
+  </si>
+  <si>
+    <t>fragments/resources-sidenav</t>
+  </si>
+  <si>
+    <t>resources-sidenav</t>
+  </si>
+  <si>
+    <t>2026-10-29T00:58:29.131Z</t>
+  </si>
+  <si>
+    <t>https://www.sfu.ca/research/researcher-resources/resources/research-facilities.html</t>
+  </si>
+  <si>
+    <t>resources/research-facilities.report.json</t>
+  </si>
+  <si>
+    <t>resources/research-facilities</t>
+  </si>
+  <si>
+    <t>resources</t>
+  </si>
+  <si>
+    <t>2026-10-29T00:58:37.859Z</t>
   </si>
   <si>
     <t>templates/landing-page.report.json</t>
@@ -124,7 +151,7 @@
     <t>landing-page</t>
   </si>
   <si>
-    <t>2026-10-28T07:31:46.139Z</t>
+    <t>2026-10-29T00:32:30.001Z</t>
   </si>
   <si>
     <t>templates/programs.report.json</t>
@@ -136,7 +163,19 @@
     <t>programs-template</t>
   </si>
   <si>
-    <t>2026-10-29T00:30:19.873Z</t>
+    <t>2026-10-29T00:49:33.239Z</t>
+  </si>
+  <si>
+    <t>templates/resources.report.json</t>
+  </si>
+  <si>
+    <t>templates/resources</t>
+  </si>
+  <si>
+    <t>resources-template</t>
+  </si>
+  <si>
+    <t>2026-10-29T00:58:47.210Z</t>
   </si>
 </sst>
 </file>
@@ -525,13 +564,13 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:I9"/>
+  <dimension ref="A1:I12"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
-    <col min="1" max="1" width="40" customWidth="1"/>
-    <col min="3" max="3" width="28" customWidth="1"/>
+    <col min="1" max="1" width="43" customWidth="1"/>
+    <col min="3" max="3" width="31" customWidth="1"/>
     <col min="4" max="4" width="10" customWidth="1"/>
-    <col min="6" max="6" width="19" customWidth="1"/>
+    <col min="6" max="6" width="20" customWidth="1"/>
     <col min="7" max="7" width="26" customWidth="1"/>
     <col min="8" max="8" width="25" customWidth="1"/>
     <col min="9" max="9" width="50" customWidth="1"/>
@@ -571,7 +610,7 @@
         <v>9</v>
       </c>
       <c r="B2">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="C2" t="s">
         <v>10</v>
@@ -766,36 +805,123 @@
         <v>11</v>
       </c>
       <c r="I8" t="s">
-        <v>14</v>
+        <v>38</v>
       </c>
     </row>
     <row r="9" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
+        <v>39</v>
+      </c>
+      <c r="B9" t="s">
+        <v>11</v>
+      </c>
+      <c r="C9" t="s">
+        <v>40</v>
+      </c>
+      <c r="D9" t="s">
+        <v>11</v>
+      </c>
+      <c r="E9" t="s">
+        <v>12</v>
+      </c>
+      <c r="F9" t="s">
+        <v>41</v>
+      </c>
+      <c r="G9" t="s">
+        <v>42</v>
+      </c>
+      <c r="H9" t="s">
+        <v>11</v>
+      </c>
+      <c r="I9" t="s">
         <v>38</v>
       </c>
-      <c r="B9" t="s">
-        <v>11</v>
-      </c>
-      <c r="C9" t="s">
-        <v>39</v>
-      </c>
-      <c r="D9" t="s">
-        <v>11</v>
-      </c>
-      <c r="E9" t="s">
-        <v>12</v>
-      </c>
-      <c r="F9" t="s">
-        <v>40</v>
-      </c>
-      <c r="G9" t="s">
-        <v>41</v>
-      </c>
-      <c r="H9" t="s">
-        <v>11</v>
-      </c>
-      <c r="I9" t="s">
+    </row>
+    <row r="10" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
+        <v>43</v>
+      </c>
+      <c r="B10" t="s">
+        <v>11</v>
+      </c>
+      <c r="C10" t="s">
+        <v>44</v>
+      </c>
+      <c r="D10" t="s">
+        <v>11</v>
+      </c>
+      <c r="E10" t="s">
+        <v>12</v>
+      </c>
+      <c r="F10" t="s">
+        <v>45</v>
+      </c>
+      <c r="G10" t="s">
+        <v>46</v>
+      </c>
+      <c r="H10" t="s">
+        <v>11</v>
+      </c>
+      <c r="I10" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="11" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
+        <v>47</v>
+      </c>
+      <c r="B11" t="s">
+        <v>11</v>
+      </c>
+      <c r="C11" t="s">
+        <v>48</v>
+      </c>
+      <c r="D11" t="s">
+        <v>11</v>
+      </c>
+      <c r="E11" t="s">
+        <v>12</v>
+      </c>
+      <c r="F11" t="s">
+        <v>49</v>
+      </c>
+      <c r="G11" t="s">
+        <v>50</v>
+      </c>
+      <c r="H11" t="s">
+        <v>11</v>
+      </c>
+      <c r="I11" t="s">
         <v>29</v>
+      </c>
+    </row>
+    <row r="12" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A12" t="s">
+        <v>51</v>
+      </c>
+      <c r="B12" t="s">
+        <v>11</v>
+      </c>
+      <c r="C12" t="s">
+        <v>52</v>
+      </c>
+      <c r="D12" t="s">
+        <v>11</v>
+      </c>
+      <c r="E12" t="s">
+        <v>12</v>
+      </c>
+      <c r="F12" t="s">
+        <v>53</v>
+      </c>
+      <c r="G12" t="s">
+        <v>54</v>
+      </c>
+      <c r="H12" t="s">
+        <v>11</v>
+      </c>
+      <c r="I12" t="s">
+        <v>38</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Add global region personalisation (| region | canada/usa/international | block row)
- scripts.js: region row on any block is removed and the block kept only for
  the visitor's region (?region= override, default canada); runs before blocks load
- Region promo fragment importer and block library examples

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/tools/importer/reports/import-block-library.report.xlsx
+++ b/tools/importer/reports/import-block-library.report.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="106" uniqueCount="55">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="148" uniqueCount="72">
   <si>
     <t>_reportFile</t>
   </si>
@@ -22,6 +22,9 @@
     <t>path</t>
   </si>
   <si>
+    <t>region</t>
+  </si>
+  <si>
     <t>sections</t>
   </si>
   <si>
@@ -52,7 +55,7 @@
     <t>success</t>
   </si>
   <si>
-    <t>2026-10-29T00:58:57.058Z</t>
+    <t>2026-10-29T02:18:45.651Z</t>
   </si>
   <si>
     <t>https://www.sfu.ca/</t>
@@ -97,7 +100,7 @@
     <t>programs</t>
   </si>
   <si>
-    <t>2026-10-29T00:49:24.817Z</t>
+    <t>2026-10-29T01:19:49.954Z</t>
   </si>
   <si>
     <t>https://www.sfu.ca/beedie/programs/undergraduate/bba-major/program.html</t>
@@ -115,6 +118,54 @@
     <t>2026-10-29T00:31:18.120Z</t>
   </si>
   <si>
+    <t>fragments/promo-canada.report.json</t>
+  </si>
+  <si>
+    <t>fragments/promo-canada</t>
+  </si>
+  <si>
+    <t>canada</t>
+  </si>
+  <si>
+    <t>region-promo</t>
+  </si>
+  <si>
+    <t>2026-10-29T02:18:22.145Z</t>
+  </si>
+  <si>
+    <t>https://www.sfu.ca/?promo=canada</t>
+  </si>
+  <si>
+    <t>fragments/promo-international.report.json</t>
+  </si>
+  <si>
+    <t>fragments/promo-international</t>
+  </si>
+  <si>
+    <t>international</t>
+  </si>
+  <si>
+    <t>2026-10-29T02:18:35.317Z</t>
+  </si>
+  <si>
+    <t>https://www.sfu.ca/?promo=international</t>
+  </si>
+  <si>
+    <t>fragments/promo-usa.report.json</t>
+  </si>
+  <si>
+    <t>fragments/promo-usa</t>
+  </si>
+  <si>
+    <t>usa</t>
+  </si>
+  <si>
+    <t>2026-10-29T02:18:28.462Z</t>
+  </si>
+  <si>
+    <t>https://www.sfu.ca/?promo=usa</t>
+  </si>
+  <si>
     <t>fragments/resources-sidenav.report.json</t>
   </si>
   <si>
@@ -139,7 +190,7 @@
     <t>resources</t>
   </si>
   <si>
-    <t>2026-10-29T00:58:37.859Z</t>
+    <t>2026-10-29T01:20:07.922Z</t>
   </si>
   <si>
     <t>templates/landing-page.report.json</t>
@@ -163,7 +214,7 @@
     <t>programs-template</t>
   </si>
   <si>
-    <t>2026-10-29T00:49:33.239Z</t>
+    <t>2026-10-29T01:19:59.428Z</t>
   </si>
   <si>
     <t>templates/resources.report.json</t>
@@ -175,7 +226,7 @@
     <t>resources-template</t>
   </si>
   <si>
-    <t>2026-10-29T00:58:47.210Z</t>
+    <t>2026-10-29T01:20:16.898Z</t>
   </si>
 </sst>
 </file>
@@ -564,19 +615,20 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:I12"/>
+  <dimension ref="A1:J15"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="43" customWidth="1"/>
     <col min="3" max="3" width="31" customWidth="1"/>
-    <col min="4" max="4" width="10" customWidth="1"/>
-    <col min="6" max="6" width="20" customWidth="1"/>
-    <col min="7" max="7" width="26" customWidth="1"/>
-    <col min="8" max="8" width="25" customWidth="1"/>
-    <col min="9" max="9" width="50" customWidth="1"/>
+    <col min="4" max="4" width="15" customWidth="1"/>
+    <col min="5" max="5" width="10" customWidth="1"/>
+    <col min="7" max="7" width="20" customWidth="1"/>
+    <col min="8" max="8" width="26" customWidth="1"/>
+    <col min="9" max="9" width="25" customWidth="1"/>
+    <col min="10" max="10" width="50" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" s="1" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:10" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -604,83 +656,92 @@
       <c r="I1" s="1" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="2" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="J1" s="1" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="2" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="B2">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="C2" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="D2" t="s">
+        <v>12</v>
+      </c>
+      <c r="E2" t="s">
+        <v>12</v>
+      </c>
+      <c r="F2" t="s">
+        <v>13</v>
+      </c>
+      <c r="G2" t="s">
         <v>11</v>
       </c>
-      <c r="E2" t="s">
-        <v>12</v>
-      </c>
-      <c r="F2" t="s">
-        <v>10</v>
-      </c>
-      <c r="G2" t="s">
-        <v>13</v>
-      </c>
       <c r="H2" t="s">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="I2" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="3" spans="1:9" x14ac:dyDescent="0.25">
+        <v>12</v>
+      </c>
+      <c r="J2" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="3" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="B3" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="C3" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="D3" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="E3" t="s">
         <v>12</v>
       </c>
       <c r="F3" t="s">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="G3" t="s">
         <v>17</v>
       </c>
       <c r="H3" t="s">
+        <v>18</v>
+      </c>
+      <c r="I3" t="s">
+        <v>12</v>
+      </c>
+      <c r="J3" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="4" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>19</v>
+      </c>
+      <c r="B4" t="s">
+        <v>12</v>
+      </c>
+      <c r="C4" t="s">
+        <v>20</v>
+      </c>
+      <c r="D4" t="s">
+        <v>12</v>
+      </c>
+      <c r="E4">
         <v>11</v>
       </c>
-      <c r="I3" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="4" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A4" t="s">
-        <v>18</v>
-      </c>
-      <c r="B4" t="s">
-        <v>11</v>
-      </c>
-      <c r="C4" t="s">
-        <v>19</v>
-      </c>
-      <c r="D4">
-        <v>11</v>
-      </c>
-      <c r="E4" t="s">
-        <v>12</v>
-      </c>
       <c r="F4" t="s">
-        <v>20</v>
+        <v>13</v>
       </c>
       <c r="G4" t="s">
         <v>21</v>
@@ -689,243 +750,366 @@
         <v>22</v>
       </c>
       <c r="I4" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="5" spans="1:9" x14ac:dyDescent="0.25">
+        <v>23</v>
+      </c>
+      <c r="J4" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="5" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="B5" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="C5" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="D5" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="E5" t="s">
         <v>12</v>
       </c>
       <c r="F5" t="s">
-        <v>24</v>
+        <v>13</v>
       </c>
       <c r="G5" t="s">
         <v>25</v>
       </c>
       <c r="H5" t="s">
-        <v>11</v>
+        <v>26</v>
       </c>
       <c r="I5" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="6" spans="1:9" x14ac:dyDescent="0.25">
+        <v>12</v>
+      </c>
+      <c r="J5" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="6" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="B6" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="C6" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="D6" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="E6" t="s">
         <v>12</v>
       </c>
       <c r="F6" t="s">
-        <v>27</v>
+        <v>13</v>
       </c>
       <c r="G6" t="s">
         <v>28</v>
       </c>
       <c r="H6" t="s">
-        <v>11</v>
+        <v>29</v>
       </c>
       <c r="I6" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="7" spans="1:9" x14ac:dyDescent="0.25">
+        <v>12</v>
+      </c>
+      <c r="J6" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="7" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="B7" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="C7" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="D7" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="E7" t="s">
         <v>12</v>
       </c>
       <c r="F7" t="s">
-        <v>32</v>
+        <v>13</v>
       </c>
       <c r="G7" t="s">
         <v>33</v>
       </c>
       <c r="H7" t="s">
-        <v>11</v>
+        <v>34</v>
       </c>
       <c r="I7" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="8" spans="1:9" x14ac:dyDescent="0.25">
+        <v>12</v>
+      </c>
+      <c r="J7" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="8" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="B8" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="C8" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="D8" t="s">
-        <v>11</v>
+        <v>37</v>
       </c>
       <c r="E8" t="s">
         <v>12</v>
       </c>
       <c r="F8" t="s">
-        <v>36</v>
+        <v>13</v>
       </c>
       <c r="G8" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="H8" t="s">
-        <v>11</v>
+        <v>39</v>
       </c>
       <c r="I8" t="s">
+        <v>12</v>
+      </c>
+      <c r="J8" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="9" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>41</v>
+      </c>
+      <c r="B9" t="s">
+        <v>12</v>
+      </c>
+      <c r="C9" t="s">
+        <v>42</v>
+      </c>
+      <c r="D9" t="s">
+        <v>43</v>
+      </c>
+      <c r="E9" t="s">
+        <v>12</v>
+      </c>
+      <c r="F9" t="s">
+        <v>13</v>
+      </c>
+      <c r="G9" t="s">
         <v>38</v>
       </c>
-    </row>
-    <row r="9" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A9" t="s">
-        <v>39</v>
-      </c>
-      <c r="B9" t="s">
-        <v>11</v>
-      </c>
-      <c r="C9" t="s">
-        <v>40</v>
-      </c>
-      <c r="D9" t="s">
-        <v>11</v>
-      </c>
-      <c r="E9" t="s">
-        <v>12</v>
-      </c>
-      <c r="F9" t="s">
-        <v>41</v>
-      </c>
-      <c r="G9" t="s">
-        <v>42</v>
-      </c>
       <c r="H9" t="s">
-        <v>11</v>
+        <v>44</v>
       </c>
       <c r="I9" t="s">
+        <v>12</v>
+      </c>
+      <c r="J9" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="10" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
+        <v>46</v>
+      </c>
+      <c r="B10" t="s">
+        <v>12</v>
+      </c>
+      <c r="C10" t="s">
+        <v>47</v>
+      </c>
+      <c r="D10" t="s">
+        <v>48</v>
+      </c>
+      <c r="E10" t="s">
+        <v>12</v>
+      </c>
+      <c r="F10" t="s">
+        <v>13</v>
+      </c>
+      <c r="G10" t="s">
         <v>38</v>
       </c>
-    </row>
-    <row r="10" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A10" t="s">
-        <v>43</v>
-      </c>
-      <c r="B10" t="s">
-        <v>11</v>
-      </c>
-      <c r="C10" t="s">
-        <v>44</v>
-      </c>
-      <c r="D10" t="s">
-        <v>11</v>
-      </c>
-      <c r="E10" t="s">
-        <v>12</v>
-      </c>
-      <c r="F10" t="s">
-        <v>45</v>
-      </c>
-      <c r="G10" t="s">
-        <v>46</v>
-      </c>
       <c r="H10" t="s">
-        <v>11</v>
+        <v>49</v>
       </c>
       <c r="I10" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="11" spans="1:9" x14ac:dyDescent="0.25">
+        <v>12</v>
+      </c>
+      <c r="J10" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="11" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>47</v>
+        <v>51</v>
       </c>
       <c r="B11" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="C11" t="s">
-        <v>48</v>
+        <v>52</v>
       </c>
       <c r="D11" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="E11" t="s">
         <v>12</v>
       </c>
       <c r="F11" t="s">
-        <v>49</v>
+        <v>13</v>
       </c>
       <c r="G11" t="s">
-        <v>50</v>
+        <v>53</v>
       </c>
       <c r="H11" t="s">
-        <v>11</v>
+        <v>54</v>
       </c>
       <c r="I11" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="12" spans="1:9" x14ac:dyDescent="0.25">
+        <v>12</v>
+      </c>
+      <c r="J11" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="12" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>51</v>
+        <v>56</v>
       </c>
       <c r="B12" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="C12" t="s">
-        <v>52</v>
+        <v>57</v>
       </c>
       <c r="D12" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="E12" t="s">
         <v>12</v>
       </c>
       <c r="F12" t="s">
-        <v>53</v>
+        <v>13</v>
       </c>
       <c r="G12" t="s">
-        <v>54</v>
+        <v>58</v>
       </c>
       <c r="H12" t="s">
-        <v>11</v>
+        <v>59</v>
       </c>
       <c r="I12" t="s">
-        <v>38</v>
+        <v>12</v>
+      </c>
+      <c r="J12" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="13" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A13" t="s">
+        <v>60</v>
+      </c>
+      <c r="B13" t="s">
+        <v>12</v>
+      </c>
+      <c r="C13" t="s">
+        <v>61</v>
+      </c>
+      <c r="D13" t="s">
+        <v>12</v>
+      </c>
+      <c r="E13" t="s">
+        <v>12</v>
+      </c>
+      <c r="F13" t="s">
+        <v>13</v>
+      </c>
+      <c r="G13" t="s">
+        <v>62</v>
+      </c>
+      <c r="H13" t="s">
+        <v>63</v>
+      </c>
+      <c r="I13" t="s">
+        <v>12</v>
+      </c>
+      <c r="J13" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="14" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A14" t="s">
+        <v>64</v>
+      </c>
+      <c r="B14" t="s">
+        <v>12</v>
+      </c>
+      <c r="C14" t="s">
+        <v>65</v>
+      </c>
+      <c r="D14" t="s">
+        <v>12</v>
+      </c>
+      <c r="E14" t="s">
+        <v>12</v>
+      </c>
+      <c r="F14" t="s">
+        <v>13</v>
+      </c>
+      <c r="G14" t="s">
+        <v>66</v>
+      </c>
+      <c r="H14" t="s">
+        <v>67</v>
+      </c>
+      <c r="I14" t="s">
+        <v>12</v>
+      </c>
+      <c r="J14" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="15" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A15" t="s">
+        <v>68</v>
+      </c>
+      <c r="B15" t="s">
+        <v>12</v>
+      </c>
+      <c r="C15" t="s">
+        <v>69</v>
+      </c>
+      <c r="D15" t="s">
+        <v>12</v>
+      </c>
+      <c r="E15" t="s">
+        <v>12</v>
+      </c>
+      <c r="F15" t="s">
+        <v>13</v>
+      </c>
+      <c r="G15" t="s">
+        <v>70</v>
+      </c>
+      <c r="H15" t="s">
+        <v>71</v>
+      </c>
+      <c r="I15" t="s">
+        <v>12</v>
+      </c>
+      <c r="J15" t="s">
+        <v>55</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:I1"/>
+  <autoFilter ref="A1:J1"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
 </worksheet>

</xml_diff>

<commit_message>
Homepage: region-tailored Visit panel and Stats for canada, usa, international
- lib/sfu-regional.js: regional copy and the region-row helper
- Block library keeps the unrestricted Visit panel and Stats examples

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/tools/importer/reports/import-block-library.report.xlsx
+++ b/tools/importer/reports/import-block-library.report.xlsx
@@ -55,7 +55,7 @@
     <t>success</t>
   </si>
   <si>
-    <t>2026-10-29T02:18:45.651Z</t>
+    <t>2026-10-29T02:25:34.189Z</t>
   </si>
   <si>
     <t>https://www.sfu.ca/</t>
@@ -79,7 +79,7 @@
     <t>homepage</t>
   </si>
   <si>
-    <t>2026-10-28T07:31:25.455Z</t>
+    <t>2026-10-29T02:25:23.458Z</t>
   </si>
   <si>
     <t>Simon Fraser University</t>

</xml_diff>

<commit_message>
Add DA Library importers: block sample pages and library templates
- lib/sfu-library-examples.js: shared block/variant examples for /block-library and DA Library
- import-library-docs.js: one sample page per block under /docs/library/blocks (named variants + descriptions)
- Template importers: ?target=library writes to /docs/library/templates

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/tools/importer/reports/import-block-library.report.xlsx
+++ b/tools/importer/reports/import-block-library.report.xlsx
@@ -55,7 +55,7 @@
     <t>success</t>
   </si>
   <si>
-    <t>2026-10-29T02:25:34.189Z</t>
+    <t>2026-10-29T03:05:30.105Z</t>
   </si>
   <si>
     <t>https://www.sfu.ca/</t>
@@ -79,7 +79,7 @@
     <t>homepage</t>
   </si>
   <si>
-    <t>2026-10-29T02:25:23.458Z</t>
+    <t>2026-10-29T02:41:05.901Z</t>
   </si>
   <si>
     <t>Simon Fraser University</t>

</xml_diff>

<commit_message>
Link sidenavs to migrated DA pages; templates only in the DA Library
- Page map: BBA Program and Curriculum now resolve to /programs/bba-major/*
- BBA importer writes to /programs/bba-major/program
- Library examples link to the migrated pages
- Template importers write only to /docs/library/templates

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/tools/importer/reports/import-block-library.report.xlsx
+++ b/tools/importer/reports/import-block-library.report.xlsx
@@ -11,11 +11,14 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="148" uniqueCount="72">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="306" uniqueCount="135">
   <si>
     <t>_reportFile</t>
   </si>
   <si>
+    <t>doc</t>
+  </si>
+  <si>
     <t>entries</t>
   </si>
   <si>
@@ -46,16 +49,16 @@
     <t>block-library.report.json</t>
   </si>
   <si>
+    <t/>
+  </si>
+  <si>
     <t>block-library</t>
   </si>
   <si>
-    <t/>
-  </si>
-  <si>
     <t>success</t>
   </si>
   <si>
-    <t>2026-10-29T03:05:30.105Z</t>
+    <t>2026-10-29T15:33:53.284Z</t>
   </si>
   <si>
     <t>https://www.sfu.ca/</t>
@@ -115,7 +118,7 @@
     <t>programs-sidenav</t>
   </si>
   <si>
-    <t>2026-10-29T00:31:18.120Z</t>
+    <t>2026-10-29T15:33:43.066Z</t>
   </si>
   <si>
     <t>fragments/promo-canada.report.json</t>
@@ -227,6 +230,192 @@
   </si>
   <si>
     <t>2026-10-29T01:20:16.898Z</t>
+  </si>
+  <si>
+    <t>docs/library/blocks/accordion.report.json</t>
+  </si>
+  <si>
+    <t>accordion</t>
+  </si>
+  <si>
+    <t>docs/library/blocks/accordion</t>
+  </si>
+  <si>
+    <t>library-doc</t>
+  </si>
+  <si>
+    <t>2026-10-29T03:06:08.512Z</t>
+  </si>
+  <si>
+    <t>https://www.sfu.ca/?libdoc=accordion</t>
+  </si>
+  <si>
+    <t>docs/library/blocks/cards.report.json</t>
+  </si>
+  <si>
+    <t>cards</t>
+  </si>
+  <si>
+    <t>docs/library/blocks/cards</t>
+  </si>
+  <si>
+    <t>2026-10-29T03:05:48.263Z</t>
+  </si>
+  <si>
+    <t>https://www.sfu.ca/?libdoc=cards</t>
+  </si>
+  <si>
+    <t>docs/library/blocks/columns.report.json</t>
+  </si>
+  <si>
+    <t>columns</t>
+  </si>
+  <si>
+    <t>docs/library/blocks/columns</t>
+  </si>
+  <si>
+    <t>2026-10-29T03:05:55.952Z</t>
+  </si>
+  <si>
+    <t>https://www.sfu.ca/?libdoc=columns</t>
+  </si>
+  <si>
+    <t>docs/library/blocks/facilities.report.json</t>
+  </si>
+  <si>
+    <t>facilities</t>
+  </si>
+  <si>
+    <t>docs/library/blocks/facilities</t>
+  </si>
+  <si>
+    <t>2026-10-29T03:06:22.317Z</t>
+  </si>
+  <si>
+    <t>https://www.sfu.ca/?libdoc=facilities</t>
+  </si>
+  <si>
+    <t>docs/library/blocks/fragment.report.json</t>
+  </si>
+  <si>
+    <t>fragment</t>
+  </si>
+  <si>
+    <t>docs/library/blocks/fragment</t>
+  </si>
+  <si>
+    <t>2026-10-29T03:06:28.382Z</t>
+  </si>
+  <si>
+    <t>https://www.sfu.ca/?libdoc=fragment</t>
+  </si>
+  <si>
+    <t>docs/library/blocks/hero.report.json</t>
+  </si>
+  <si>
+    <t>hero</t>
+  </si>
+  <si>
+    <t>docs/library/blocks/hero</t>
+  </si>
+  <si>
+    <t>2026-10-29T03:05:40.236Z</t>
+  </si>
+  <si>
+    <t>https://www.sfu.ca/?libdoc=hero</t>
+  </si>
+  <si>
+    <t>docs/library/blocks/region.report.json</t>
+  </si>
+  <si>
+    <t>docs/library/blocks/region</t>
+  </si>
+  <si>
+    <t>2026-10-29T03:06:34.590Z</t>
+  </si>
+  <si>
+    <t>https://www.sfu.ca/?libdoc=region</t>
+  </si>
+  <si>
+    <t>docs/library/blocks/section-metadata.report.json</t>
+  </si>
+  <si>
+    <t>section-metadata</t>
+  </si>
+  <si>
+    <t>docs/library/blocks/section-metadata</t>
+  </si>
+  <si>
+    <t>2026-10-29T03:06:40.889Z</t>
+  </si>
+  <si>
+    <t>https://www.sfu.ca/?libdoc=section-metadata</t>
+  </si>
+  <si>
+    <t>docs/library/blocks/sidenav.report.json</t>
+  </si>
+  <si>
+    <t>sidenav</t>
+  </si>
+  <si>
+    <t>docs/library/blocks/sidenav</t>
+  </si>
+  <si>
+    <t>2026-10-29T03:06:16.382Z</t>
+  </si>
+  <si>
+    <t>https://www.sfu.ca/?libdoc=sidenav</t>
+  </si>
+  <si>
+    <t>docs/library/blocks/stats.report.json</t>
+  </si>
+  <si>
+    <t>stats</t>
+  </si>
+  <si>
+    <t>docs/library/blocks/stats</t>
+  </si>
+  <si>
+    <t>2026-10-29T03:06:02.703Z</t>
+  </si>
+  <si>
+    <t>https://www.sfu.ca/?libdoc=stats</t>
+  </si>
+  <si>
+    <t>docs/library/templates/landing-page.report.json</t>
+  </si>
+  <si>
+    <t>docs/library/templates/landing-page</t>
+  </si>
+  <si>
+    <t>2026-10-29T03:06:50.552Z</t>
+  </si>
+  <si>
+    <t>https://www.sfu.ca/?target=library</t>
+  </si>
+  <si>
+    <t>docs/library/templates/programs.report.json</t>
+  </si>
+  <si>
+    <t>docs/library/templates/programs</t>
+  </si>
+  <si>
+    <t>2026-10-29T03:07:00.204Z</t>
+  </si>
+  <si>
+    <t>https://www.sfu.ca/beedie/programs/undergraduate/bba-major/program.html?target=library</t>
+  </si>
+  <si>
+    <t>docs/library/templates/resources.report.json</t>
+  </si>
+  <si>
+    <t>docs/library/templates/resources</t>
+  </si>
+  <si>
+    <t>2026-10-29T03:07:09.328Z</t>
+  </si>
+  <si>
+    <t>https://www.sfu.ca/research/researcher-resources/resources/research-facilities.html?target=library</t>
   </si>
 </sst>
 </file>
@@ -615,20 +804,21 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:J15"/>
+  <dimension ref="A1:K28"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
-    <col min="1" max="1" width="43" customWidth="1"/>
-    <col min="3" max="3" width="31" customWidth="1"/>
-    <col min="4" max="4" width="15" customWidth="1"/>
-    <col min="5" max="5" width="10" customWidth="1"/>
-    <col min="7" max="7" width="20" customWidth="1"/>
-    <col min="8" max="8" width="26" customWidth="1"/>
-    <col min="9" max="9" width="25" customWidth="1"/>
-    <col min="10" max="10" width="50" customWidth="1"/>
+    <col min="1" max="1" width="50" customWidth="1"/>
+    <col min="2" max="2" width="18" customWidth="1"/>
+    <col min="4" max="4" width="38" customWidth="1"/>
+    <col min="5" max="5" width="15" customWidth="1"/>
+    <col min="6" max="6" width="10" customWidth="1"/>
+    <col min="8" max="8" width="20" customWidth="1"/>
+    <col min="9" max="9" width="26" customWidth="1"/>
+    <col min="10" max="10" width="25" customWidth="1"/>
+    <col min="11" max="11" width="50" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" s="1" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:11" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -659,92 +849,101 @@
       <c r="J1" s="1" t="s">
         <v>9</v>
       </c>
-    </row>
-    <row r="2" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="K1" s="1" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="2" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>10</v>
-      </c>
-      <c r="B2">
+        <v>11</v>
+      </c>
+      <c r="B2" t="s">
+        <v>12</v>
+      </c>
+      <c r="C2">
         <v>20</v>
       </c>
-      <c r="C2" t="s">
-        <v>11</v>
-      </c>
       <c r="D2" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="E2" t="s">
         <v>12</v>
       </c>
       <c r="F2" t="s">
+        <v>12</v>
+      </c>
+      <c r="G2" t="s">
+        <v>14</v>
+      </c>
+      <c r="H2" t="s">
         <v>13</v>
       </c>
-      <c r="G2" t="s">
-        <v>11</v>
-      </c>
-      <c r="H2" t="s">
-        <v>14</v>
-      </c>
       <c r="I2" t="s">
-        <v>12</v>
+        <v>15</v>
       </c>
       <c r="J2" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="3" spans="1:10" x14ac:dyDescent="0.25">
+        <v>12</v>
+      </c>
+      <c r="K2" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="3" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="B3" t="s">
         <v>12</v>
       </c>
       <c r="C3" t="s">
-        <v>17</v>
+        <v>12</v>
       </c>
       <c r="D3" t="s">
-        <v>12</v>
+        <v>18</v>
       </c>
       <c r="E3" t="s">
         <v>12</v>
       </c>
       <c r="F3" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="G3" t="s">
-        <v>17</v>
+        <v>14</v>
       </c>
       <c r="H3" t="s">
         <v>18</v>
       </c>
       <c r="I3" t="s">
-        <v>12</v>
+        <v>19</v>
       </c>
       <c r="J3" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="4" spans="1:10" x14ac:dyDescent="0.25">
+        <v>12</v>
+      </c>
+      <c r="K3" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="4" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="B4" t="s">
         <v>12</v>
       </c>
       <c r="C4" t="s">
-        <v>20</v>
+        <v>12</v>
       </c>
       <c r="D4" t="s">
-        <v>12</v>
-      </c>
-      <c r="E4">
+        <v>21</v>
+      </c>
+      <c r="E4" t="s">
+        <v>12</v>
+      </c>
+      <c r="F4">
         <v>11</v>
       </c>
-      <c r="F4" t="s">
-        <v>13</v>
-      </c>
       <c r="G4" t="s">
-        <v>21</v>
+        <v>14</v>
       </c>
       <c r="H4" t="s">
         <v>22</v>
@@ -753,363 +952,854 @@
         <v>23</v>
       </c>
       <c r="J4" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="5" spans="1:10" x14ac:dyDescent="0.25">
+        <v>24</v>
+      </c>
+      <c r="K4" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="5" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="B5" t="s">
         <v>12</v>
       </c>
       <c r="C5" t="s">
-        <v>25</v>
+        <v>12</v>
       </c>
       <c r="D5" t="s">
-        <v>12</v>
+        <v>26</v>
       </c>
       <c r="E5" t="s">
         <v>12</v>
       </c>
       <c r="F5" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="G5" t="s">
-        <v>25</v>
+        <v>14</v>
       </c>
       <c r="H5" t="s">
         <v>26</v>
       </c>
       <c r="I5" t="s">
-        <v>12</v>
+        <v>27</v>
       </c>
       <c r="J5" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="6" spans="1:10" x14ac:dyDescent="0.25">
+        <v>12</v>
+      </c>
+      <c r="K5" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="6" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="B6" t="s">
         <v>12</v>
       </c>
       <c r="C6" t="s">
-        <v>28</v>
+        <v>12</v>
       </c>
       <c r="D6" t="s">
-        <v>12</v>
+        <v>29</v>
       </c>
       <c r="E6" t="s">
         <v>12</v>
       </c>
       <c r="F6" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="G6" t="s">
-        <v>28</v>
+        <v>14</v>
       </c>
       <c r="H6" t="s">
         <v>29</v>
       </c>
       <c r="I6" t="s">
-        <v>12</v>
+        <v>30</v>
       </c>
       <c r="J6" t="s">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="7" spans="1:10" x14ac:dyDescent="0.25">
+        <v>12</v>
+      </c>
+      <c r="K6" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="7" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="B7" t="s">
         <v>12</v>
       </c>
       <c r="C7" t="s">
-        <v>32</v>
+        <v>12</v>
       </c>
       <c r="D7" t="s">
-        <v>12</v>
+        <v>33</v>
       </c>
       <c r="E7" t="s">
         <v>12</v>
       </c>
       <c r="F7" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="G7" t="s">
-        <v>33</v>
+        <v>14</v>
       </c>
       <c r="H7" t="s">
         <v>34</v>
       </c>
       <c r="I7" t="s">
-        <v>12</v>
+        <v>35</v>
       </c>
       <c r="J7" t="s">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="8" spans="1:10" x14ac:dyDescent="0.25">
+        <v>12</v>
+      </c>
+      <c r="K7" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="8" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="B8" t="s">
         <v>12</v>
       </c>
       <c r="C8" t="s">
-        <v>36</v>
+        <v>12</v>
       </c>
       <c r="D8" t="s">
         <v>37</v>
       </c>
       <c r="E8" t="s">
-        <v>12</v>
+        <v>38</v>
       </c>
       <c r="F8" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="G8" t="s">
-        <v>38</v>
+        <v>14</v>
       </c>
       <c r="H8" t="s">
         <v>39</v>
       </c>
       <c r="I8" t="s">
-        <v>12</v>
+        <v>40</v>
       </c>
       <c r="J8" t="s">
-        <v>40</v>
-      </c>
-    </row>
-    <row r="9" spans="1:10" x14ac:dyDescent="0.25">
+        <v>12</v>
+      </c>
+      <c r="K8" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="9" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="B9" t="s">
         <v>12</v>
       </c>
       <c r="C9" t="s">
-        <v>42</v>
+        <v>12</v>
       </c>
       <c r="D9" t="s">
         <v>43</v>
       </c>
       <c r="E9" t="s">
-        <v>12</v>
+        <v>44</v>
       </c>
       <c r="F9" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="G9" t="s">
-        <v>38</v>
+        <v>14</v>
       </c>
       <c r="H9" t="s">
-        <v>44</v>
+        <v>39</v>
       </c>
       <c r="I9" t="s">
-        <v>12</v>
+        <v>45</v>
       </c>
       <c r="J9" t="s">
-        <v>45</v>
-      </c>
-    </row>
-    <row r="10" spans="1:10" x14ac:dyDescent="0.25">
+        <v>12</v>
+      </c>
+      <c r="K9" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="10" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="B10" t="s">
         <v>12</v>
       </c>
       <c r="C10" t="s">
-        <v>47</v>
+        <v>12</v>
       </c>
       <c r="D10" t="s">
         <v>48</v>
       </c>
       <c r="E10" t="s">
-        <v>12</v>
+        <v>49</v>
       </c>
       <c r="F10" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="G10" t="s">
-        <v>38</v>
+        <v>14</v>
       </c>
       <c r="H10" t="s">
-        <v>49</v>
+        <v>39</v>
       </c>
       <c r="I10" t="s">
-        <v>12</v>
+        <v>50</v>
       </c>
       <c r="J10" t="s">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="11" spans="1:10" x14ac:dyDescent="0.25">
+        <v>12</v>
+      </c>
+      <c r="K10" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="11" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="B11" t="s">
         <v>12</v>
       </c>
       <c r="C11" t="s">
-        <v>52</v>
+        <v>12</v>
       </c>
       <c r="D11" t="s">
-        <v>12</v>
+        <v>53</v>
       </c>
       <c r="E11" t="s">
         <v>12</v>
       </c>
       <c r="F11" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="G11" t="s">
-        <v>53</v>
+        <v>14</v>
       </c>
       <c r="H11" t="s">
         <v>54</v>
       </c>
       <c r="I11" t="s">
-        <v>12</v>
+        <v>55</v>
       </c>
       <c r="J11" t="s">
-        <v>55</v>
-      </c>
-    </row>
-    <row r="12" spans="1:10" x14ac:dyDescent="0.25">
+        <v>12</v>
+      </c>
+      <c r="K11" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="12" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="B12" t="s">
         <v>12</v>
       </c>
       <c r="C12" t="s">
-        <v>57</v>
+        <v>12</v>
       </c>
       <c r="D12" t="s">
-        <v>12</v>
+        <v>58</v>
       </c>
       <c r="E12" t="s">
         <v>12</v>
       </c>
       <c r="F12" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="G12" t="s">
-        <v>58</v>
+        <v>14</v>
       </c>
       <c r="H12" t="s">
         <v>59</v>
       </c>
       <c r="I12" t="s">
-        <v>12</v>
+        <v>60</v>
       </c>
       <c r="J12" t="s">
-        <v>55</v>
-      </c>
-    </row>
-    <row r="13" spans="1:10" x14ac:dyDescent="0.25">
+        <v>12</v>
+      </c>
+      <c r="K12" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="13" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="B13" t="s">
         <v>12</v>
       </c>
       <c r="C13" t="s">
-        <v>61</v>
+        <v>12</v>
       </c>
       <c r="D13" t="s">
-        <v>12</v>
+        <v>62</v>
       </c>
       <c r="E13" t="s">
         <v>12</v>
       </c>
       <c r="F13" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="G13" t="s">
-        <v>62</v>
+        <v>14</v>
       </c>
       <c r="H13" t="s">
         <v>63</v>
       </c>
       <c r="I13" t="s">
-        <v>12</v>
+        <v>64</v>
       </c>
       <c r="J13" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="14" spans="1:10" x14ac:dyDescent="0.25">
+        <v>12</v>
+      </c>
+      <c r="K13" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="14" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="B14" t="s">
         <v>12</v>
       </c>
       <c r="C14" t="s">
-        <v>65</v>
+        <v>12</v>
       </c>
       <c r="D14" t="s">
-        <v>12</v>
+        <v>66</v>
       </c>
       <c r="E14" t="s">
         <v>12</v>
       </c>
       <c r="F14" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="G14" t="s">
-        <v>66</v>
+        <v>14</v>
       </c>
       <c r="H14" t="s">
         <v>67</v>
       </c>
       <c r="I14" t="s">
-        <v>12</v>
+        <v>68</v>
       </c>
       <c r="J14" t="s">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="15" spans="1:10" x14ac:dyDescent="0.25">
+        <v>12</v>
+      </c>
+      <c r="K14" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="15" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="B15" t="s">
         <v>12</v>
       </c>
       <c r="C15" t="s">
-        <v>69</v>
+        <v>12</v>
       </c>
       <c r="D15" t="s">
-        <v>12</v>
+        <v>70</v>
       </c>
       <c r="E15" t="s">
         <v>12</v>
       </c>
       <c r="F15" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="G15" t="s">
-        <v>70</v>
+        <v>14</v>
       </c>
       <c r="H15" t="s">
         <v>71</v>
       </c>
       <c r="I15" t="s">
-        <v>12</v>
+        <v>72</v>
       </c>
       <c r="J15" t="s">
-        <v>55</v>
+        <v>12</v>
+      </c>
+      <c r="K15" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="16" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A16" t="s">
+        <v>73</v>
+      </c>
+      <c r="B16" t="s">
+        <v>74</v>
+      </c>
+      <c r="C16" t="s">
+        <v>12</v>
+      </c>
+      <c r="D16" t="s">
+        <v>75</v>
+      </c>
+      <c r="E16" t="s">
+        <v>12</v>
+      </c>
+      <c r="F16" t="s">
+        <v>12</v>
+      </c>
+      <c r="G16" t="s">
+        <v>14</v>
+      </c>
+      <c r="H16" t="s">
+        <v>76</v>
+      </c>
+      <c r="I16" t="s">
+        <v>77</v>
+      </c>
+      <c r="J16" t="s">
+        <v>12</v>
+      </c>
+      <c r="K16" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="17" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A17" t="s">
+        <v>79</v>
+      </c>
+      <c r="B17" t="s">
+        <v>80</v>
+      </c>
+      <c r="C17" t="s">
+        <v>12</v>
+      </c>
+      <c r="D17" t="s">
+        <v>81</v>
+      </c>
+      <c r="E17" t="s">
+        <v>12</v>
+      </c>
+      <c r="F17" t="s">
+        <v>12</v>
+      </c>
+      <c r="G17" t="s">
+        <v>14</v>
+      </c>
+      <c r="H17" t="s">
+        <v>76</v>
+      </c>
+      <c r="I17" t="s">
+        <v>82</v>
+      </c>
+      <c r="J17" t="s">
+        <v>12</v>
+      </c>
+      <c r="K17" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="18" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A18" t="s">
+        <v>84</v>
+      </c>
+      <c r="B18" t="s">
+        <v>85</v>
+      </c>
+      <c r="C18" t="s">
+        <v>12</v>
+      </c>
+      <c r="D18" t="s">
+        <v>86</v>
+      </c>
+      <c r="E18" t="s">
+        <v>12</v>
+      </c>
+      <c r="F18" t="s">
+        <v>12</v>
+      </c>
+      <c r="G18" t="s">
+        <v>14</v>
+      </c>
+      <c r="H18" t="s">
+        <v>76</v>
+      </c>
+      <c r="I18" t="s">
+        <v>87</v>
+      </c>
+      <c r="J18" t="s">
+        <v>12</v>
+      </c>
+      <c r="K18" t="s">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="19" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A19" t="s">
+        <v>89</v>
+      </c>
+      <c r="B19" t="s">
+        <v>90</v>
+      </c>
+      <c r="C19" t="s">
+        <v>12</v>
+      </c>
+      <c r="D19" t="s">
+        <v>91</v>
+      </c>
+      <c r="E19" t="s">
+        <v>12</v>
+      </c>
+      <c r="F19" t="s">
+        <v>12</v>
+      </c>
+      <c r="G19" t="s">
+        <v>14</v>
+      </c>
+      <c r="H19" t="s">
+        <v>76</v>
+      </c>
+      <c r="I19" t="s">
+        <v>92</v>
+      </c>
+      <c r="J19" t="s">
+        <v>12</v>
+      </c>
+      <c r="K19" t="s">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="20" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A20" t="s">
+        <v>94</v>
+      </c>
+      <c r="B20" t="s">
+        <v>95</v>
+      </c>
+      <c r="C20" t="s">
+        <v>12</v>
+      </c>
+      <c r="D20" t="s">
+        <v>96</v>
+      </c>
+      <c r="E20" t="s">
+        <v>12</v>
+      </c>
+      <c r="F20" t="s">
+        <v>12</v>
+      </c>
+      <c r="G20" t="s">
+        <v>14</v>
+      </c>
+      <c r="H20" t="s">
+        <v>76</v>
+      </c>
+      <c r="I20" t="s">
+        <v>97</v>
+      </c>
+      <c r="J20" t="s">
+        <v>12</v>
+      </c>
+      <c r="K20" t="s">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="21" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A21" t="s">
+        <v>99</v>
+      </c>
+      <c r="B21" t="s">
+        <v>100</v>
+      </c>
+      <c r="C21" t="s">
+        <v>12</v>
+      </c>
+      <c r="D21" t="s">
+        <v>101</v>
+      </c>
+      <c r="E21" t="s">
+        <v>12</v>
+      </c>
+      <c r="F21" t="s">
+        <v>12</v>
+      </c>
+      <c r="G21" t="s">
+        <v>14</v>
+      </c>
+      <c r="H21" t="s">
+        <v>76</v>
+      </c>
+      <c r="I21" t="s">
+        <v>102</v>
+      </c>
+      <c r="J21" t="s">
+        <v>12</v>
+      </c>
+      <c r="K21" t="s">
+        <v>103</v>
+      </c>
+    </row>
+    <row r="22" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A22" t="s">
+        <v>104</v>
+      </c>
+      <c r="B22" t="s">
+        <v>4</v>
+      </c>
+      <c r="C22" t="s">
+        <v>12</v>
+      </c>
+      <c r="D22" t="s">
+        <v>105</v>
+      </c>
+      <c r="E22" t="s">
+        <v>12</v>
+      </c>
+      <c r="F22" t="s">
+        <v>12</v>
+      </c>
+      <c r="G22" t="s">
+        <v>14</v>
+      </c>
+      <c r="H22" t="s">
+        <v>76</v>
+      </c>
+      <c r="I22" t="s">
+        <v>106</v>
+      </c>
+      <c r="J22" t="s">
+        <v>12</v>
+      </c>
+      <c r="K22" t="s">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="23" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A23" t="s">
+        <v>108</v>
+      </c>
+      <c r="B23" t="s">
+        <v>109</v>
+      </c>
+      <c r="C23" t="s">
+        <v>12</v>
+      </c>
+      <c r="D23" t="s">
+        <v>110</v>
+      </c>
+      <c r="E23" t="s">
+        <v>12</v>
+      </c>
+      <c r="F23" t="s">
+        <v>12</v>
+      </c>
+      <c r="G23" t="s">
+        <v>14</v>
+      </c>
+      <c r="H23" t="s">
+        <v>76</v>
+      </c>
+      <c r="I23" t="s">
+        <v>111</v>
+      </c>
+      <c r="J23" t="s">
+        <v>12</v>
+      </c>
+      <c r="K23" t="s">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="24" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A24" t="s">
+        <v>113</v>
+      </c>
+      <c r="B24" t="s">
+        <v>114</v>
+      </c>
+      <c r="C24" t="s">
+        <v>12</v>
+      </c>
+      <c r="D24" t="s">
+        <v>115</v>
+      </c>
+      <c r="E24" t="s">
+        <v>12</v>
+      </c>
+      <c r="F24" t="s">
+        <v>12</v>
+      </c>
+      <c r="G24" t="s">
+        <v>14</v>
+      </c>
+      <c r="H24" t="s">
+        <v>76</v>
+      </c>
+      <c r="I24" t="s">
+        <v>116</v>
+      </c>
+      <c r="J24" t="s">
+        <v>12</v>
+      </c>
+      <c r="K24" t="s">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="25" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A25" t="s">
+        <v>118</v>
+      </c>
+      <c r="B25" t="s">
+        <v>119</v>
+      </c>
+      <c r="C25" t="s">
+        <v>12</v>
+      </c>
+      <c r="D25" t="s">
+        <v>120</v>
+      </c>
+      <c r="E25" t="s">
+        <v>12</v>
+      </c>
+      <c r="F25" t="s">
+        <v>12</v>
+      </c>
+      <c r="G25" t="s">
+        <v>14</v>
+      </c>
+      <c r="H25" t="s">
+        <v>76</v>
+      </c>
+      <c r="I25" t="s">
+        <v>121</v>
+      </c>
+      <c r="J25" t="s">
+        <v>12</v>
+      </c>
+      <c r="K25" t="s">
+        <v>122</v>
+      </c>
+    </row>
+    <row r="26" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A26" t="s">
+        <v>123</v>
+      </c>
+      <c r="B26" t="s">
+        <v>12</v>
+      </c>
+      <c r="C26" t="s">
+        <v>12</v>
+      </c>
+      <c r="D26" t="s">
+        <v>124</v>
+      </c>
+      <c r="E26" t="s">
+        <v>12</v>
+      </c>
+      <c r="F26" t="s">
+        <v>12</v>
+      </c>
+      <c r="G26" t="s">
+        <v>14</v>
+      </c>
+      <c r="H26" t="s">
+        <v>63</v>
+      </c>
+      <c r="I26" t="s">
+        <v>125</v>
+      </c>
+      <c r="J26" t="s">
+        <v>12</v>
+      </c>
+      <c r="K26" t="s">
+        <v>126</v>
+      </c>
+    </row>
+    <row r="27" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A27" t="s">
+        <v>127</v>
+      </c>
+      <c r="B27" t="s">
+        <v>12</v>
+      </c>
+      <c r="C27" t="s">
+        <v>12</v>
+      </c>
+      <c r="D27" t="s">
+        <v>128</v>
+      </c>
+      <c r="E27" t="s">
+        <v>12</v>
+      </c>
+      <c r="F27" t="s">
+        <v>12</v>
+      </c>
+      <c r="G27" t="s">
+        <v>14</v>
+      </c>
+      <c r="H27" t="s">
+        <v>67</v>
+      </c>
+      <c r="I27" t="s">
+        <v>129</v>
+      </c>
+      <c r="J27" t="s">
+        <v>12</v>
+      </c>
+      <c r="K27" t="s">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="28" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A28" t="s">
+        <v>131</v>
+      </c>
+      <c r="B28" t="s">
+        <v>12</v>
+      </c>
+      <c r="C28" t="s">
+        <v>12</v>
+      </c>
+      <c r="D28" t="s">
+        <v>132</v>
+      </c>
+      <c r="E28" t="s">
+        <v>12</v>
+      </c>
+      <c r="F28" t="s">
+        <v>12</v>
+      </c>
+      <c r="G28" t="s">
+        <v>14</v>
+      </c>
+      <c r="H28" t="s">
+        <v>71</v>
+      </c>
+      <c r="I28" t="s">
+        <v>133</v>
+      </c>
+      <c r="J28" t="s">
+        <v>12</v>
+      </c>
+      <c r="K28" t="s">
+        <v>134</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:J1"/>
+  <autoFilter ref="A1:K1"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
 </worksheet>

</xml_diff>

<commit_message>
Add Teaser block from the Figma Content Teaser
Background image with overlay, optional pre-heading, heading, intro and
buttons. Options: top/bottom, center/right, wide, focus-left/focus-right
and link (whole banner linked, hover overlay and red bar). Layout switches
on the teaser's own width (576px container query). Adds Teaser samples to
the DA Library doc (/docs/library/blocks/teaser) and the block library page.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/tools/importer/reports/import-block-library.report.xlsx
+++ b/tools/importer/reports/import-block-library.report.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="306" uniqueCount="135">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="317" uniqueCount="140">
   <si>
     <t>_reportFile</t>
   </si>
@@ -58,7 +58,7 @@
     <t>success</t>
   </si>
   <si>
-    <t>2026-10-29T15:33:53.284Z</t>
+    <t>2026-10-29T17:09:19.723Z</t>
   </si>
   <si>
     <t>https://www.sfu.ca/</t>
@@ -259,7 +259,7 @@
     <t>docs/library/blocks/cards</t>
   </si>
   <si>
-    <t>2026-10-29T03:05:48.263Z</t>
+    <t>2026-10-29T15:34:11.022Z</t>
   </si>
   <si>
     <t>https://www.sfu.ca/?libdoc=cards</t>
@@ -361,7 +361,7 @@
     <t>docs/library/blocks/sidenav</t>
   </si>
   <si>
-    <t>2026-10-29T03:06:16.382Z</t>
+    <t>2026-10-29T15:34:02.889Z</t>
   </si>
   <si>
     <t>https://www.sfu.ca/?libdoc=sidenav</t>
@@ -380,6 +380,21 @@
   </si>
   <si>
     <t>https://www.sfu.ca/?libdoc=stats</t>
+  </si>
+  <si>
+    <t>docs/library/blocks/teaser.report.json</t>
+  </si>
+  <si>
+    <t>teaser</t>
+  </si>
+  <si>
+    <t>docs/library/blocks/teaser</t>
+  </si>
+  <si>
+    <t>2026-10-29T17:07:54.223Z</t>
+  </si>
+  <si>
+    <t>https://www.sfu.ca/?libdoc=teaser</t>
   </si>
   <si>
     <t>docs/library/templates/landing-page.report.json</t>
@@ -804,7 +819,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:K28"/>
+  <dimension ref="A1:K29"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="50" customWidth="1"/>
@@ -861,7 +876,7 @@
         <v>12</v>
       </c>
       <c r="C2">
-        <v>20</v>
+        <v>23</v>
       </c>
       <c r="D2" t="s">
         <v>13</v>
@@ -1698,13 +1713,13 @@
         <v>123</v>
       </c>
       <c r="B26" t="s">
-        <v>12</v>
+        <v>124</v>
       </c>
       <c r="C26" t="s">
         <v>12</v>
       </c>
       <c r="D26" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="E26" t="s">
         <v>12</v>
@@ -1716,21 +1731,21 @@
         <v>14</v>
       </c>
       <c r="H26" t="s">
-        <v>63</v>
+        <v>76</v>
       </c>
       <c r="I26" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="J26" t="s">
         <v>12</v>
       </c>
       <c r="K26" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
     </row>
     <row r="27" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="B27" t="s">
         <v>12</v>
@@ -1739,7 +1754,7 @@
         <v>12</v>
       </c>
       <c r="D27" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="E27" t="s">
         <v>12</v>
@@ -1751,21 +1766,21 @@
         <v>14</v>
       </c>
       <c r="H27" t="s">
-        <v>67</v>
+        <v>63</v>
       </c>
       <c r="I27" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="J27" t="s">
         <v>12</v>
       </c>
       <c r="K27" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
     </row>
     <row r="28" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="B28" t="s">
         <v>12</v>
@@ -1774,7 +1789,7 @@
         <v>12</v>
       </c>
       <c r="D28" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="E28" t="s">
         <v>12</v>
@@ -1786,16 +1801,51 @@
         <v>14</v>
       </c>
       <c r="H28" t="s">
+        <v>67</v>
+      </c>
+      <c r="I28" t="s">
+        <v>134</v>
+      </c>
+      <c r="J28" t="s">
+        <v>12</v>
+      </c>
+      <c r="K28" t="s">
+        <v>135</v>
+      </c>
+    </row>
+    <row r="29" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A29" t="s">
+        <v>136</v>
+      </c>
+      <c r="B29" t="s">
+        <v>12</v>
+      </c>
+      <c r="C29" t="s">
+        <v>12</v>
+      </c>
+      <c r="D29" t="s">
+        <v>137</v>
+      </c>
+      <c r="E29" t="s">
+        <v>12</v>
+      </c>
+      <c r="F29" t="s">
+        <v>12</v>
+      </c>
+      <c r="G29" t="s">
+        <v>14</v>
+      </c>
+      <c r="H29" t="s">
         <v>71</v>
       </c>
-      <c r="I28" t="s">
-        <v>133</v>
-      </c>
-      <c r="J28" t="s">
-        <v>12</v>
-      </c>
-      <c r="K28" t="s">
-        <v>134</v>
+      <c r="I29" t="s">
+        <v>138</v>
+      </c>
+      <c r="J29" t="s">
+        <v>12</v>
+      </c>
+      <c r="K29" t="s">
+        <v>139</v>
       </c>
     </row>
   </sheetData>

</xml_diff>